<commit_message>
stock update+lazy loading for images
</commit_message>
<xml_diff>
--- a/data/stock.xlsx
+++ b/data/stock.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\blocks\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B7CCB09-05D3-4908-8739-2F99A060ECD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06CC5F2-4140-4631-ACCE-095CEBA56303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4035" yWindow="825" windowWidth="21600" windowHeight="11250" xr2:uid="{FC0CBB84-858B-49F6-BA69-44D83C89F7C4}"/>
   </bookViews>
@@ -4648,7 +4648,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -4686,9 +4686,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5182,7 +5179,7 @@
         <v>1305</v>
       </c>
       <c r="B3" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3">
         <v>260</v>
@@ -5199,7 +5196,7 @@
         <v>1457</v>
       </c>
       <c r="B4" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3">
         <v>450</v>
@@ -5250,7 +5247,7 @@
         <v>1372</v>
       </c>
       <c r="B7" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="3">
         <v>260</v>
@@ -5542,7 +5539,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="3">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>1504</v>
@@ -6304,7 +6301,7 @@
         <v>22</v>
       </c>
       <c r="B69" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C69" s="3">
         <v>180</v>
@@ -6338,7 +6335,7 @@
         <v>1118</v>
       </c>
       <c r="B71" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C71" s="3">
         <v>180</v>
@@ -6355,7 +6352,7 @@
         <v>493</v>
       </c>
       <c r="B72" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C72" s="3">
         <v>180</v>
@@ -8225,7 +8222,7 @@
         <v>1142</v>
       </c>
       <c r="B182" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C182" s="3">
         <v>280</v>
@@ -8837,7 +8834,7 @@
         <v>34</v>
       </c>
       <c r="B218" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C218" s="3">
         <v>260</v>
@@ -8990,7 +8987,7 @@
         <v>1373</v>
       </c>
       <c r="B227" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C227" s="3">
         <v>300</v>
@@ -9109,7 +9106,7 @@
         <v>399</v>
       </c>
       <c r="B234" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C234" s="3">
         <v>220</v>
@@ -9262,7 +9259,7 @@
         <v>1454</v>
       </c>
       <c r="B243" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C243" s="3">
         <v>260</v>
@@ -9840,7 +9837,7 @@
         <v>1378</v>
       </c>
       <c r="B277" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C277" s="3">
         <v>280</v>
@@ -14413,7 +14410,7 @@
         <v>167</v>
       </c>
       <c r="B546" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C546" s="3">
         <v>260</v>
@@ -17770,7 +17767,7 @@
       <c r="D743" s="4" t="s">
         <v>1512</v>
       </c>
-      <c r="E743" s="16" t="s">
+      <c r="E743" s="6" t="s">
         <v>1332</v>
       </c>
     </row>
@@ -17787,7 +17784,7 @@
       <c r="D744" s="4" t="s">
         <v>1513</v>
       </c>
-      <c r="E744" s="16" t="s">
+      <c r="E744" s="6" t="s">
         <v>1332</v>
       </c>
     </row>
@@ -17804,7 +17801,7 @@
       <c r="D745" s="4" t="s">
         <v>1514</v>
       </c>
-      <c r="E745" s="16" t="s">
+      <c r="E745" s="6" t="s">
         <v>1332</v>
       </c>
     </row>
@@ -17821,7 +17818,7 @@
       <c r="D746" s="4" t="s">
         <v>1482</v>
       </c>
-      <c r="E746" s="16" t="s">
+      <c r="E746" s="6" t="s">
         <v>1324</v>
       </c>
     </row>
@@ -17838,7 +17835,7 @@
       <c r="D747" s="4" t="s">
         <v>1484</v>
       </c>
-      <c r="E747" s="16" t="s">
+      <c r="E747" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17855,7 +17852,7 @@
       <c r="D748" s="4" t="s">
         <v>1486</v>
       </c>
-      <c r="E748" s="16" t="s">
+      <c r="E748" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17872,7 +17869,7 @@
       <c r="D749" s="4" t="s">
         <v>1487</v>
       </c>
-      <c r="E749" s="16" t="s">
+      <c r="E749" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17889,7 +17886,7 @@
       <c r="D750" s="4" t="s">
         <v>1488</v>
       </c>
-      <c r="E750" s="16" t="s">
+      <c r="E750" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17906,7 +17903,7 @@
       <c r="D751" s="4" t="s">
         <v>1489</v>
       </c>
-      <c r="E751" s="16" t="s">
+      <c r="E751" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17923,7 +17920,7 @@
       <c r="D752" s="4" t="s">
         <v>1490</v>
       </c>
-      <c r="E752" s="16" t="s">
+      <c r="E752" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17940,7 +17937,7 @@
       <c r="D753" s="4" t="s">
         <v>1491</v>
       </c>
-      <c r="E753" s="16" t="s">
+      <c r="E753" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17957,7 +17954,7 @@
       <c r="D754" s="4" t="s">
         <v>1492</v>
       </c>
-      <c r="E754" s="16" t="s">
+      <c r="E754" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17974,7 +17971,7 @@
       <c r="D755" s="4" t="s">
         <v>1493</v>
       </c>
-      <c r="E755" s="16" t="s">
+      <c r="E755" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -17991,7 +17988,7 @@
       <c r="D756" s="4" t="s">
         <v>1483</v>
       </c>
-      <c r="E756" s="16" t="s">
+      <c r="E756" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -18008,7 +18005,7 @@
       <c r="D757" s="4" t="s">
         <v>1494</v>
       </c>
-      <c r="E757" s="16" t="s">
+      <c r="E757" s="6" t="s">
         <v>174</v>
       </c>
     </row>
@@ -18025,7 +18022,7 @@
       <c r="D758" s="4" t="s">
         <v>1495</v>
       </c>
-      <c r="E758" s="16" t="s">
+      <c r="E758" s="6" t="s">
         <v>174</v>
       </c>
     </row>

</xml_diff>